<commit_message>
Refresh README with synthetic GIF workflows and architecture visuals
</commit_message>
<xml_diff>
--- a/docs/examples/harbor-path/exports/tracked-flows.xlsx
+++ b/docs/examples/harbor-path/exports/tracked-flows.xlsx
@@ -1135,7 +1135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1206,12 +1206,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>远帆供应</t>
+          <t>松原项目</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SYN-F001</t>
+          <t>SYN-G001</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1220,273 +1220,33 @@
         </is>
       </c>
       <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
         <v>3</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>437501.00</t>
         </is>
       </c>
-      <c r="G2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>437501.00</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>875002.00</t>
-        </is>
-      </c>
       <c r="J2" s="1" t="n">
-        <v>46271.60416666666</v>
+        <v>46276.47916666666</v>
       </c>
       <c r="K2" s="1" t="n">
         <v>46278.5625</v>
       </c>
       <c r="L2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>云杉工坊</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>SYN-A001</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>480000.00</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>480000.00</t>
-        </is>
-      </c>
-      <c r="J3" s="1" t="n">
-        <v>46267.4375</v>
-      </c>
-      <c r="K3" s="1" t="n">
-        <v>46267.4375</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>松原项目</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>SYN-G001</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>3</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>437501.00</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>437501.00</t>
-        </is>
-      </c>
-      <c r="J4" s="1" t="n">
-        <v>46276.47916666666</v>
-      </c>
-      <c r="K4" s="1" t="n">
-        <v>46278.5625</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>青禾工程</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>SYN-C001</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>162500.50</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>182500.50</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>345001.00</t>
-        </is>
-      </c>
-      <c r="J5" s="1" t="n">
-        <v>46268.47916666666</v>
-      </c>
-      <c r="K5" s="1" t="n">
-        <v>46275.4375</v>
-      </c>
-      <c r="L5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>汀兰材料</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>SYN-E001</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>165000.50</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>175000.50</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>340001.00</t>
-        </is>
-      </c>
-      <c r="J6" s="1" t="n">
-        <v>46270.5625</v>
-      </c>
-      <c r="K6" s="1" t="n">
-        <v>46273.6875</v>
-      </c>
-      <c r="L6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>岚山物流</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>SYN-D001</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>110000.00</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>120000.00</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>230000.00</t>
-        </is>
-      </c>
-      <c r="J7" s="1" t="n">
-        <v>46269.52083333334</v>
-      </c>
-      <c r="K7" s="1" t="n">
-        <v>46272.64583333334</v>
-      </c>
-      <c r="L7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>